<commit_message>
fix time and clear deadline
</commit_message>
<xml_diff>
--- a/dianguc_data.xlsx
+++ b/dianguc_data.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -876,9 +876,17 @@
         <v>sai</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>sai</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix stop bot in battle
</commit_message>
<xml_diff>
--- a/dianguc_data.xlsx
+++ b/dianguc_data.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -883,10 +883,21 @@
       <c r="B29" t="str">
         <v>sai</v>
       </c>
+      <c r="C29" t="str">
+        <v>đúng</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>sai</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>